<commit_message>
Working version of feed-forward connections
In this version, miniature network is 500
e4scnn1a cells.
It produces a nice curve of turning angle
and f1/evoked rates.
</commit_message>
<xml_diff>
--- a/base_props/V1model_seed_file_miniature.xlsx
+++ b/base_props/V1model_seed_file_miniature.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10912"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11010"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shinya.ito/wsdata/glif_builder/base_props/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{876A4A9E-4533-F742-A59F-6D787185A5D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BE7C775-2213-BD41-97DC-CAB8C80D2EF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26940" yWindow="17000" windowWidth="25600" windowHeight="15540" xr2:uid="{CFFEA874-25CC-4540-BE90-5AB415846019}"/>
+    <workbookView xWindow="17380" yWindow="12200" windowWidth="25600" windowHeight="15540" xr2:uid="{CFFEA874-25CC-4540-BE90-5AB415846019}"/>
   </bookViews>
   <sheets>
     <sheet name="cell_models" sheetId="1" r:id="rId1"/>
@@ -35,20 +35,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="44">
-  <si>
-    <t>e4Nr5a1</t>
-  </si>
-  <si>
-    <t>e4Rorb</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>e4Scnn1a</t>
   </si>
   <si>
-    <t>e4other</t>
-  </si>
-  <si>
     <t>VisL4</t>
   </si>
   <si>
@@ -115,22 +106,10 @@
     <t>positive</t>
   </si>
   <si>
-    <t>negative</t>
-  </si>
-  <si>
     <t>cre_line</t>
   </si>
   <si>
-    <t>Nr5a1</t>
-  </si>
-  <si>
-    <t>Rorb</t>
-  </si>
-  <si>
     <t>Scnn1a</t>
-  </si>
-  <si>
-    <t>Nr5a1,Rorb,Scnn1a</t>
   </si>
   <si>
     <t>pop_name</t>
@@ -528,7 +507,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06D17F6F-74AA-824C-8392-CC22C78F6ABE}">
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.33203125" customWidth="1"/>
@@ -549,375 +528,210 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G1" t="s">
         <v>32</v>
       </c>
-      <c r="C1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1" t="s">
+        <v>31</v>
+      </c>
+      <c r="J1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" t="s">
+        <v>17</v>
+      </c>
+      <c r="M1" t="s">
+        <v>28</v>
+      </c>
+      <c r="N1" t="s">
+        <v>29</v>
+      </c>
+      <c r="O1" t="s">
         <v>27</v>
-      </c>
-      <c r="F1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H1" t="s">
-        <v>37</v>
-      </c>
-      <c r="I1" t="s">
-        <v>38</v>
-      </c>
-      <c r="J1" t="s">
-        <v>23</v>
-      </c>
-      <c r="K1" t="s">
-        <v>19</v>
-      </c>
-      <c r="L1" t="s">
-        <v>20</v>
-      </c>
-      <c r="M1" t="s">
-        <v>35</v>
-      </c>
-      <c r="N1" t="s">
-        <v>36</v>
-      </c>
-      <c r="O1" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D2" t="str">
-        <f t="shared" ref="D2:D5" si="0">LEFT(B2, 1)</f>
+        <f t="shared" ref="D2" si="0">LEFT(B2, 1)</f>
         <v>e</v>
       </c>
       <c r="E2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="H2">
-        <f>$C$21</f>
-        <v>357</v>
+        <f>$C$36</f>
+        <v>0</v>
       </c>
       <c r="I2">
-        <f>$C$22</f>
-        <v>505</v>
+        <f>$C$37</f>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>0.12</v>
+        <v>0.3</v>
       </c>
       <c r="K2">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="L2">
         <v>0.11</v>
       </c>
       <c r="M2">
-        <f t="shared" ref="M2:M5" si="1">ROUND(K2*J2*IF(EXACT(D2,"i"), L2, 1-L2), 0)</f>
-        <v>214</v>
+        <f t="shared" ref="M2" si="1">ROUND(K2*J2*IF(EXACT(D2,"i"), L2, 1-L2), 0)</f>
+        <v>134</v>
       </c>
       <c r="N2">
-        <f>ROUND(M2/$J$20*$K$20, 0)</f>
-        <v>741</v>
+        <f>ROUND(M2/$J$14*$K$14, 0)</f>
+        <v>464</v>
       </c>
       <c r="O2">
-        <f t="shared" ref="O2:O5" si="2">SUM(M2:N2)</f>
-        <v>955</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3">
+        <f t="shared" ref="O2" si="2">SUM(M2:N2)</f>
+        <v>598</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12" t="s">
+        <v>4</v>
+      </c>
+      <c r="I12" t="s">
+        <v>12</v>
+      </c>
+      <c r="J12" t="s">
+        <v>15</v>
+      </c>
+      <c r="K12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" t="str">
-        <f t="shared" si="0"/>
-        <v>e</v>
-      </c>
-      <c r="E3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F3" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3">
-        <f>$C$21</f>
+      <c r="B13">
+        <v>50</v>
+      </c>
+      <c r="C13">
+        <f>SUM($B$13:$B13)</f>
+        <v>50</v>
+      </c>
+      <c r="I13" t="s">
+        <v>13</v>
+      </c>
+      <c r="J13">
+        <v>0.4</v>
+      </c>
+      <c r="K13">
+        <v>0.84499999999999997</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14">
+        <v>119</v>
+      </c>
+      <c r="C14">
+        <f>SUM($B$13:$B14)</f>
+        <v>169</v>
+      </c>
+      <c r="I14" t="s">
+        <v>14</v>
+      </c>
+      <c r="J14" s="1">
+        <f>J13^2*PI()</f>
+        <v>0.50265482457436694</v>
+      </c>
+      <c r="K14" s="1">
+        <f>K13^2*PI() - J13^2*PI()</f>
+        <v>1.7405208699050847</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15">
+        <v>188</v>
+      </c>
+      <c r="C15">
+        <f>SUM($B$13:$B15)</f>
         <v>357</v>
       </c>
-      <c r="I3">
-        <f>$C$22</f>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16">
+        <v>148</v>
+      </c>
+      <c r="C16">
+        <f>SUM($B$13:$B16)</f>
         <v>505</v>
       </c>
-      <c r="J3">
-        <v>0.26</v>
-      </c>
-      <c r="K3">
-        <v>2000</v>
-      </c>
-      <c r="L3">
-        <v>0.11</v>
-      </c>
-      <c r="M3">
-        <f t="shared" si="1"/>
-        <v>463</v>
-      </c>
-      <c r="N3">
-        <f>ROUND(M3/$J$20*$K$20, 0)</f>
-        <v>1603</v>
-      </c>
-      <c r="O3">
-        <f t="shared" si="2"/>
-        <v>2066</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>7</v>
-      </c>
-      <c r="B4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4" t="str">
-        <f t="shared" si="0"/>
-        <v>e</v>
-      </c>
-      <c r="E4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F4" t="s">
-        <v>25</v>
-      </c>
-      <c r="H4">
-        <f>$C$21</f>
-        <v>357</v>
-      </c>
-      <c r="I4">
-        <f>$C$22</f>
-        <v>505</v>
-      </c>
-      <c r="J4">
-        <v>0.3</v>
-      </c>
-      <c r="K4">
-        <v>2000</v>
-      </c>
-      <c r="L4">
-        <v>0.11</v>
-      </c>
-      <c r="M4">
-        <f t="shared" si="1"/>
-        <v>534</v>
-      </c>
-      <c r="N4">
-        <f>ROUND(M4/$J$20*$K$20, 0)</f>
-        <v>1849</v>
-      </c>
-      <c r="O4">
-        <f t="shared" si="2"/>
-        <v>2383</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" t="str">
-        <f t="shared" si="0"/>
-        <v>e</v>
-      </c>
-      <c r="E5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5" t="s">
-        <v>26</v>
-      </c>
-      <c r="H5">
-        <f>$C$21</f>
-        <v>357</v>
-      </c>
-      <c r="I5">
-        <f>$C$22</f>
-        <v>505</v>
-      </c>
-      <c r="J5">
-        <f>1-SUM($J2:$J4)</f>
-        <v>0.32000000000000006</v>
-      </c>
-      <c r="K5">
-        <v>2000</v>
-      </c>
-      <c r="L5">
-        <v>0.11</v>
-      </c>
-      <c r="M5">
-        <f t="shared" si="1"/>
-        <v>570</v>
-      </c>
-      <c r="N5">
-        <f>ROUND(M5/$J$20*$K$20, 0)</f>
-        <v>1974</v>
-      </c>
-      <c r="O5">
-        <f t="shared" si="2"/>
-        <v>2544</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="M7">
-        <f>SUM(M2:M5)</f>
-        <v>1781</v>
-      </c>
-      <c r="N7">
-        <f>SUM(N2:N5)</f>
-        <v>6167</v>
-      </c>
-      <c r="O7">
-        <f>SUM(O2:O5)</f>
-        <v>7948</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17">
+        <v>160</v>
+      </c>
+      <c r="C17">
+        <f>SUM($B$13:$B17)</f>
+        <v>665</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>8</v>
-      </c>
-      <c r="B18" t="s">
-        <v>6</v>
-      </c>
-      <c r="C18" t="s">
-        <v>7</v>
-      </c>
-      <c r="I18" t="s">
-        <v>15</v>
-      </c>
-      <c r="J18" t="s">
-        <v>18</v>
-      </c>
-      <c r="K18" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>9</v>
-      </c>
-      <c r="B19">
-        <v>50</v>
-      </c>
-      <c r="C19">
-        <f>SUM($B$19:$B19)</f>
-        <v>50</v>
-      </c>
-      <c r="I19" t="s">
-        <v>16</v>
-      </c>
-      <c r="J19">
-        <v>0.4</v>
-      </c>
-      <c r="K19">
-        <v>0.84499999999999997</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>10</v>
-      </c>
-      <c r="B20">
-        <v>119</v>
-      </c>
-      <c r="C20">
-        <f>SUM($B$19:$B20)</f>
-        <v>169</v>
-      </c>
-      <c r="I20" t="s">
-        <v>17</v>
-      </c>
-      <c r="J20" s="1">
-        <f>J19^2*PI()</f>
-        <v>0.50265482457436694</v>
-      </c>
-      <c r="K20" s="1">
-        <f>K19^2*PI() - J19^2*PI()</f>
-        <v>1.7405208699050847</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
         <v>11</v>
       </c>
-      <c r="B21">
-        <v>188</v>
-      </c>
-      <c r="C21">
-        <f>SUM($B$19:$B21)</f>
-        <v>357</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>12</v>
-      </c>
-      <c r="B22">
-        <v>148</v>
-      </c>
-      <c r="C22">
-        <f>SUM($B$19:$B22)</f>
-        <v>505</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>13</v>
-      </c>
-      <c r="B23">
-        <v>160</v>
-      </c>
-      <c r="C23">
-        <f>SUM($B$19:$B23)</f>
-        <v>665</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>14</v>
-      </c>
-      <c r="B24">
+      <c r="B18">
         <v>164</v>
       </c>
-      <c r="C24">
-        <f>SUM($B$19:$B24)</f>
+      <c r="C18">
+        <f>SUM($B$13:$B18)</f>
         <v>829</v>
       </c>
     </row>
@@ -938,15 +752,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="B2">
         <f>845 / 100</f>
@@ -955,7 +769,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B3">
         <f>400/100</f>

</xml_diff>